<commit_message>
data(jpy): daily refresh 2026-09-09T07:30Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{BFB8B605-79B7-42F6-8E01-C24952D79392}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{6F1AC643-7EB8-4268-BEE7-70B72738D2EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46272</v>
+        <v>46273</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>129231</v>
+        <v>127935</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>24091</v>
+        <v>23239</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>105140</v>
+        <v>104696</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2633,14 +2633,14 @@
       <c r="J12" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="K12" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="L12" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="M12" s="45" t="s">
-        <v>46</v>
+      <c r="K12" s="43">
+        <v>1.0249999999999999</v>
+      </c>
+      <c r="L12" s="43">
+        <v>1.0249999999999999</v>
+      </c>
+      <c r="M12" s="45">
+        <v>1.0249999999999999</v>
       </c>
       <c r="O12" s="47"/>
       <c r="P12" s="48"/>
@@ -2682,13 +2682,13 @@
         <v>50</v>
       </c>
       <c r="K13" s="43">
-        <v>0.97</v>
+        <v>1.0249999999999999</v>
       </c>
       <c r="L13" s="43">
-        <v>0.97</v>
+        <v>1.0249999999999999</v>
       </c>
       <c r="M13" s="45">
-        <v>0.97</v>
+        <v>1.0249999999999999</v>
       </c>
       <c r="O13" s="86" t="s">
         <v>25</v>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>40943</v>
+        <v>39729</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2804,14 +2804,14 @@
       <c r="G16" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H16" s="52">
-        <v>0.97</v>
-      </c>
-      <c r="I16" s="52">
-        <v>0.97</v>
-      </c>
-      <c r="J16" s="55">
-        <v>0.97</v>
+      <c r="H16" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="I16" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="J16" s="55" t="s">
+        <v>46</v>
       </c>
       <c r="K16" s="52" t="s">
         <v>3</v>
@@ -2854,14 +2854,14 @@
       <c r="J17" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K17" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L17" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M17" s="54" t="s">
-        <v>46</v>
+      <c r="K17" s="52">
+        <v>0.98199999999999998</v>
+      </c>
+      <c r="L17" s="52">
+        <v>0.99</v>
+      </c>
+      <c r="M17" s="54">
+        <v>0.98599999999999999</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="39.9" customHeight="1">
@@ -2937,13 +2937,13 @@
         <v>46</v>
       </c>
       <c r="K19" s="43">
-        <v>0.98299999999999998</v>
+        <v>0.98099999999999998</v>
       </c>
       <c r="L19" s="43">
-        <v>1.05</v>
+        <v>1.06</v>
       </c>
       <c r="M19" s="45">
-        <v>1.0049999999999999</v>
+        <v>0.997</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2977,14 +2977,14 @@
       <c r="J20" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K20" s="52">
-        <v>1.0900000000000001</v>
-      </c>
-      <c r="L20" s="52">
-        <v>1.1299999999999999</v>
-      </c>
-      <c r="M20" s="54">
-        <v>1.117</v>
+      <c r="K20" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L20" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M20" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3018,14 +3018,14 @@
       <c r="J21" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K21" s="58">
-        <v>1.1399999999999999</v>
-      </c>
-      <c r="L21" s="58">
-        <v>1.22</v>
-      </c>
-      <c r="M21" s="60">
-        <v>1.167</v>
+      <c r="K21" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="L21" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="M21" s="60" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="39.9" customHeight="1">
@@ -3060,13 +3060,13 @@
         <v>46</v>
       </c>
       <c r="K22" s="65">
-        <v>1.3</v>
+        <v>1.26</v>
       </c>
       <c r="L22" s="65">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="M22" s="67">
-        <v>1.3</v>
+        <v>1.268</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3100,14 +3100,14 @@
       <c r="J23" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K23" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L23" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M23" s="54" t="s">
-        <v>46</v>
+      <c r="K23" s="52">
+        <v>1.5</v>
+      </c>
+      <c r="L23" s="52">
+        <v>1.5</v>
+      </c>
+      <c r="M23" s="54">
+        <v>1.5</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="39.9" customHeight="1">
@@ -3132,23 +3132,23 @@
       <c r="G24" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H24" s="52">
-        <v>1.39</v>
-      </c>
-      <c r="I24" s="52">
-        <v>1.39</v>
-      </c>
-      <c r="J24" s="55">
-        <v>1.39</v>
-      </c>
-      <c r="K24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M24" s="54" t="s">
-        <v>46</v>
+      <c r="H24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="I24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="J24" s="55" t="s">
+        <v>46</v>
+      </c>
+      <c r="K24" s="52">
+        <v>1.36</v>
+      </c>
+      <c r="L24" s="52">
+        <v>1.36</v>
+      </c>
+      <c r="M24" s="54">
+        <v>1.36</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-09-10T07:27Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{6F1AC643-7EB8-4268-BEE7-70B72738D2EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{DF7E079D-264B-4DDE-8F48-4C03A992D1B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46273</v>
+        <v>46274</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>127935</v>
+        <v>128237</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>23239</v>
+        <v>23003</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>104696</v>
+        <v>105234</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2582,7 +2582,7 @@
         <v>0.95</v>
       </c>
       <c r="I11" s="36">
-        <v>0.97799999999999998</v>
+        <v>1.03</v>
       </c>
       <c r="J11" s="39">
         <v>0.97699999999999998</v>
@@ -2633,14 +2633,14 @@
       <c r="J12" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="K12" s="43">
-        <v>1.0249999999999999</v>
-      </c>
-      <c r="L12" s="43">
-        <v>1.0249999999999999</v>
-      </c>
-      <c r="M12" s="45">
-        <v>1.0249999999999999</v>
+      <c r="K12" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="L12" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="M12" s="45" t="s">
+        <v>46</v>
       </c>
       <c r="O12" s="47"/>
       <c r="P12" s="48"/>
@@ -2681,14 +2681,14 @@
       <c r="J13" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="K13" s="43">
-        <v>1.0249999999999999</v>
-      </c>
-      <c r="L13" s="43">
-        <v>1.0249999999999999</v>
-      </c>
-      <c r="M13" s="45">
-        <v>1.0249999999999999</v>
+      <c r="K13" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="L13" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="M13" s="45" t="s">
+        <v>46</v>
       </c>
       <c r="O13" s="86" t="s">
         <v>25</v>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>39729</v>
+        <v>39777</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2854,14 +2854,14 @@
       <c r="J17" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K17" s="52">
-        <v>0.98199999999999998</v>
-      </c>
-      <c r="L17" s="52">
-        <v>0.99</v>
-      </c>
-      <c r="M17" s="54">
-        <v>0.98599999999999999</v>
+      <c r="K17" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L17" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M17" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="39.9" customHeight="1">
@@ -2895,14 +2895,14 @@
       <c r="J18" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K18" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="L18" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="M18" s="60" t="s">
-        <v>46</v>
+      <c r="K18" s="58">
+        <v>1.06</v>
+      </c>
+      <c r="L18" s="58">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="M18" s="60">
+        <v>1.099</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="39.9" customHeight="1">
@@ -2937,13 +2937,13 @@
         <v>46</v>
       </c>
       <c r="K19" s="43">
-        <v>0.98099999999999998</v>
+        <v>0.98199999999999998</v>
       </c>
       <c r="L19" s="43">
-        <v>1.06</v>
+        <v>1.1100000000000001</v>
       </c>
       <c r="M19" s="45">
-        <v>0.997</v>
+        <v>1.0089999999999999</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2977,14 +2977,14 @@
       <c r="J20" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K20" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L20" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M20" s="54" t="s">
-        <v>46</v>
+      <c r="K20" s="52">
+        <v>1.06</v>
+      </c>
+      <c r="L20" s="52">
+        <v>1.06</v>
+      </c>
+      <c r="M20" s="54">
+        <v>1.06</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3018,14 +3018,14 @@
       <c r="J21" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K21" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="L21" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="M21" s="60" t="s">
-        <v>46</v>
+      <c r="K21" s="58">
+        <v>1.35</v>
+      </c>
+      <c r="L21" s="58">
+        <v>1.35</v>
+      </c>
+      <c r="M21" s="60">
+        <v>1.35</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="39.9" customHeight="1">
@@ -3059,14 +3059,14 @@
       <c r="J22" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="K22" s="65">
-        <v>1.26</v>
-      </c>
-      <c r="L22" s="65">
-        <v>1.27</v>
-      </c>
-      <c r="M22" s="67">
-        <v>1.268</v>
+      <c r="K22" s="65" t="s">
+        <v>3</v>
+      </c>
+      <c r="L22" s="65" t="s">
+        <v>3</v>
+      </c>
+      <c r="M22" s="67" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3100,14 +3100,14 @@
       <c r="J23" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K23" s="52">
-        <v>1.5</v>
-      </c>
-      <c r="L23" s="52">
-        <v>1.5</v>
-      </c>
-      <c r="M23" s="54">
-        <v>1.5</v>
+      <c r="K23" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L23" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M23" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="39.9" customHeight="1">
@@ -3132,23 +3132,23 @@
       <c r="G24" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="I24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="J24" s="55" t="s">
-        <v>46</v>
+      <c r="H24" s="52">
+        <v>1.42</v>
+      </c>
+      <c r="I24" s="52">
+        <v>1.42</v>
+      </c>
+      <c r="J24" s="55">
+        <v>1.42</v>
       </c>
       <c r="K24" s="52">
-        <v>1.36</v>
+        <v>1.41</v>
       </c>
       <c r="L24" s="52">
-        <v>1.36</v>
+        <v>1.41</v>
       </c>
       <c r="M24" s="54">
-        <v>1.36</v>
+        <v>1.41</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily  refresh 2026-09-11T01:27Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{DF7E079D-264B-4DDE-8F48-4C03A992D1B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{05C4E2D1-309F-44FB-B53B-C2952139F314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46274</v>
+        <v>46275</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>128237</v>
+        <v>129985</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>23003</v>
+        <v>23861</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>105234</v>
+        <v>106124</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2681,14 +2681,14 @@
       <c r="J13" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="K13" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="L13" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="M13" s="45" t="s">
-        <v>46</v>
+      <c r="K13" s="43">
+        <v>0.97499999999999998</v>
+      </c>
+      <c r="L13" s="43">
+        <v>0.97499999999999998</v>
+      </c>
+      <c r="M13" s="45">
+        <v>0.97499999999999998</v>
       </c>
       <c r="O13" s="86" t="s">
         <v>25</v>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>39777</v>
+        <v>40837</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2899,10 +2899,10 @@
         <v>1.06</v>
       </c>
       <c r="L18" s="58">
-        <v>1.1000000000000001</v>
+        <v>1.08</v>
       </c>
       <c r="M18" s="60">
-        <v>1.099</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="39.9" customHeight="1">
@@ -2937,13 +2937,13 @@
         <v>46</v>
       </c>
       <c r="K19" s="43">
-        <v>0.98199999999999998</v>
+        <v>0.98099999999999998</v>
       </c>
       <c r="L19" s="43">
-        <v>1.1100000000000001</v>
+        <v>0.98099999999999998</v>
       </c>
       <c r="M19" s="45">
-        <v>1.0089999999999999</v>
+        <v>0.98099999999999998</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2977,14 +2977,14 @@
       <c r="J20" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K20" s="52">
-        <v>1.06</v>
-      </c>
-      <c r="L20" s="52">
-        <v>1.06</v>
-      </c>
-      <c r="M20" s="54">
-        <v>1.06</v>
+      <c r="K20" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L20" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M20" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3018,14 +3018,14 @@
       <c r="J21" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K21" s="58">
-        <v>1.35</v>
-      </c>
-      <c r="L21" s="58">
-        <v>1.35</v>
-      </c>
-      <c r="M21" s="60">
-        <v>1.35</v>
+      <c r="K21" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="L21" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="M21" s="60" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="39.9" customHeight="1">
@@ -3059,14 +3059,14 @@
       <c r="J22" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="K22" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="L22" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="M22" s="67" t="s">
-        <v>46</v>
+      <c r="K22" s="65">
+        <v>1.27</v>
+      </c>
+      <c r="L22" s="65">
+        <v>1.35</v>
+      </c>
+      <c r="M22" s="67">
+        <v>1.292</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3091,14 +3091,14 @@
       <c r="G23" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H23" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="I23" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="J23" s="55" t="s">
-        <v>46</v>
+      <c r="H23" s="52">
+        <v>1.37</v>
+      </c>
+      <c r="I23" s="52">
+        <v>1.37</v>
+      </c>
+      <c r="J23" s="55">
+        <v>1.37</v>
       </c>
       <c r="K23" s="52" t="s">
         <v>3</v>
@@ -3132,23 +3132,23 @@
       <c r="G24" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H24" s="52">
-        <v>1.42</v>
-      </c>
-      <c r="I24" s="52">
-        <v>1.42</v>
-      </c>
-      <c r="J24" s="55">
-        <v>1.42</v>
-      </c>
-      <c r="K24" s="52">
-        <v>1.41</v>
-      </c>
-      <c r="L24" s="52">
-        <v>1.41</v>
-      </c>
-      <c r="M24" s="54">
-        <v>1.41</v>
+      <c r="H24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="I24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="J24" s="55" t="s">
+        <v>46</v>
+      </c>
+      <c r="K24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M24" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">
@@ -3182,14 +3182,14 @@
       <c r="J25" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K25" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L25" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M25" s="54" t="s">
-        <v>46</v>
+      <c r="K25" s="52">
+        <v>1.575</v>
+      </c>
+      <c r="L25" s="52">
+        <v>1.575</v>
+      </c>
+      <c r="M25" s="54">
+        <v>1.575</v>
       </c>
     </row>
     <row r="26" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>